<commit_message>
Added uncertainty to the model predictions and the Morris sensitivity analysis. Removed the detritivore predator from the model because it is not being used in this paper.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5923F74-6286-466C-84B7-DBC7BA437A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFA2C65-4279-49A4-B48A-43BF61C2D6F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="149">
   <si>
     <t>Parameter</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>Detritivore</t>
-  </si>
-  <si>
-    <t>DetPredator</t>
   </si>
   <si>
     <t>MAT</t>
@@ -1057,7 +1054,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1089,27 +1086,24 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="42" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1559,20 +1553,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
   <dimension ref="A1:L64"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="22.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.7265625" customWidth="1"/>
+    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="13.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1580,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -1589,36 +1583,36 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D2" s="1">
         <v>0.53</v>
@@ -1633,26 +1627,26 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D3" s="1">
         <v>0.09</v>
@@ -1667,26 +1661,26 @@
         <v>1</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D4" s="1">
         <v>700</v>
@@ -1701,26 +1695,26 @@
         <v>1160</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D5" s="4">
         <f>0.00207/0.0375</f>
@@ -1730,26 +1724,26 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D6" s="4">
         <f>0.00207/0.0375</f>
@@ -1759,26 +1753,26 @@
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D7" s="4">
         <f>0.00207/0.0375</f>
@@ -1788,26 +1782,26 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D8" s="1">
         <f>0.217/365/state_variables_value!D2</f>
@@ -1823,26 +1817,26 @@
         <v>2.7906976744186045E-4</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D9" s="1">
         <v>-5.5040310000000002E-2</v>
@@ -1851,28 +1845,28 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D10" s="1">
         <v>6</v>
@@ -1885,28 +1879,28 @@
         <v>9</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D11" s="1">
         <v>0.33</v>
@@ -1921,26 +1915,26 @@
         <v>1</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D12" s="5">
         <f>D13*0.03</f>
@@ -1959,26 +1953,26 @@
         <v>17.920000000000002</v>
       </c>
       <c r="H12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D13" s="1">
         <f>336/0.75</f>
@@ -1997,26 +1991,26 @@
         <v>448</v>
       </c>
       <c r="H13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D14" s="1">
         <v>0.22</v>
@@ -2031,26 +2025,26 @@
         <v>1</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D15" s="1">
         <v>73</v>
@@ -2063,23 +2057,23 @@
         <v>78</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1">
@@ -2093,26 +2087,26 @@
         <v>8</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D17" s="1">
         <v>0</v>
@@ -2126,25 +2120,25 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D18" s="1">
         <v>26</v>
@@ -2155,22 +2149,22 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D19" s="1">
         <v>0.15</v>
@@ -2181,22 +2175,22 @@
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D20" s="1">
         <v>0.5</v>
@@ -2206,25 +2200,25 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" s="1">
         <v>1300</v>
@@ -2237,56 +2231,56 @@
         <v>1750</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D23" s="1">
         <f>1/(2.5*365*state_variables_value!D3)</f>
@@ -2296,30 +2290,30 @@
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="I23" s="1" t="s">
-        <v>123</v>
-      </c>
       <c r="J23" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" ht="16.5" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="D24" s="22">
+        <v>110</v>
+      </c>
+      <c r="D24" s="21">
         <v>8.83</v>
       </c>
       <c r="E24" s="1"/>
@@ -2330,28 +2324,28 @@
         <v>9</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D25" s="1">
         <v>0.33</v>
@@ -2366,28 +2360,28 @@
         <v>1</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D26" s="1">
         <v>177</v>
@@ -2398,28 +2392,28 @@
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -2431,15 +2425,15 @@
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D28" s="1">
         <v>0.35</v>
@@ -2449,25 +2443,25 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D29" s="1">
         <v>45</v>
@@ -2480,25 +2474,25 @@
         <v>60</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K29" s="1"/>
       <c r="L29" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1">
@@ -2512,28 +2506,28 @@
         <v>6</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K30" s="1"/>
       <c r="L30" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D31" s="6">
         <v>0.4236007</v>
@@ -2542,28 +2536,28 @@
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K31" s="1"/>
       <c r="L31" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D32" s="6">
         <v>0.4236007</v>
@@ -2572,58 +2566,58 @@
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K32" s="1"/>
       <c r="L32" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" ht="16.5" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="D33" s="22">
+        <v>110</v>
+      </c>
+      <c r="D33" s="21">
         <v>25.65</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K33" s="1"/>
       <c r="L33" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D34" s="1">
         <v>0.15</v>
@@ -2633,25 +2627,25 @@
       <c r="G34" s="1"/>
       <c r="H34" s="14"/>
       <c r="I34" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D35" s="1">
         <v>0.50930200000000003</v>
@@ -2662,26 +2656,26 @@
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I35" s="1"/>
       <c r="J35" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K35" s="1"/>
       <c r="L35" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D36" s="1">
         <v>880</v>
@@ -2696,54 +2690,54 @@
         <v>960</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I36" s="3"/>
       <c r="J36" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K36" s="1"/>
       <c r="L36" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I37" s="1"/>
       <c r="J37" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K37" s="1"/>
       <c r="L37" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D38" s="1">
         <f>0.0058/state_variables_value!D4</f>
@@ -2755,26 +2749,26 @@
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I38" s="1"/>
       <c r="J38" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K38" s="1"/>
       <c r="L38" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D39" s="1">
         <v>12</v>
@@ -2785,26 +2779,26 @@
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I39" s="1"/>
       <c r="J39" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K39" s="1"/>
       <c r="L39" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D40" s="1">
         <v>0.2</v>
@@ -2819,26 +2813,26 @@
         <v>1</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I40" s="1"/>
       <c r="J40" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K40" s="1"/>
       <c r="L40" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D41" s="1">
         <v>212</v>
@@ -2853,26 +2847,26 @@
         <v>290</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I41" s="1"/>
       <c r="J41" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K41" s="1"/>
       <c r="L41" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D42" s="1">
         <v>1428</v>
@@ -2887,26 +2881,26 @@
         <v>1481</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I42" s="1"/>
       <c r="J42" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K42" s="1"/>
       <c r="L42" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D43" s="1">
         <v>0.35</v>
@@ -2917,26 +2911,26 @@
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I43" s="1"/>
       <c r="J43" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K43" s="1"/>
       <c r="L43" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D44" s="1">
         <v>45</v>
@@ -2947,23 +2941,23 @@
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I44" s="1"/>
       <c r="J44" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K44" s="1"/>
       <c r="L44" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1">
@@ -2975,26 +2969,26 @@
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I45" s="3"/>
       <c r="J45" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K45" s="1"/>
       <c r="L45" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D46" s="1">
         <v>10.204700000000001</v>
@@ -3005,26 +2999,26 @@
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I46" s="1"/>
       <c r="J46" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D47" s="1">
         <v>10.204700000000001</v>
@@ -3035,28 +3029,28 @@
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I47" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I47" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="J47" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K47" s="1"/>
       <c r="L47" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D48" s="1">
         <v>20</v>
@@ -3067,26 +3061,26 @@
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I48" s="1"/>
       <c r="J48" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K48" s="1"/>
       <c r="L48" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D49" s="1">
         <v>0.1</v>
@@ -3097,26 +3091,26 @@
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
       <c r="H49" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I49" s="1"/>
       <c r="J49" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K49" s="1"/>
       <c r="L49" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D50" s="1">
         <v>0.5</v>
@@ -3129,28 +3123,28 @@
         <v>0.5</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K50" s="1"/>
       <c r="L50" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D51" s="7">
         <v>1410</v>
@@ -3165,28 +3159,28 @@
         <v>1450</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K51" s="1"/>
       <c r="L51" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D52" s="9">
         <v>1.384623481E-3</v>
@@ -3201,28 +3195,28 @@
         <v>1.936006955E-3</v>
       </c>
       <c r="H52" s="7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K52" s="1"/>
       <c r="L52" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D53" s="7">
         <f>0.0181818181818182/state_variables_value!D5</f>
@@ -3234,28 +3228,28 @@
       <c r="F53" s="7"/>
       <c r="G53" s="7"/>
       <c r="H53" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K53" s="1"/>
       <c r="L53" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D54" s="4">
         <v>2.7399999999999999E-5</v>
@@ -3266,28 +3260,28 @@
       <c r="F54" s="7"/>
       <c r="G54" s="7"/>
       <c r="H54" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K54" s="1"/>
       <c r="L54" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D55" s="4">
         <v>1.2999999999999999E-5</v>
@@ -3298,28 +3292,28 @@
       <c r="F55" s="7"/>
       <c r="G55" s="7"/>
       <c r="H55" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K55" s="1"/>
       <c r="L55" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D56" s="1">
         <v>12.954660000000001</v>
@@ -3330,26 +3324,26 @@
       <c r="F56" s="7"/>
       <c r="G56" s="7"/>
       <c r="H56" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I56" s="1"/>
       <c r="J56" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K56" s="1"/>
       <c r="L56" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D57" s="1">
         <v>0.17</v>
@@ -3362,28 +3356,28 @@
         <v>0.2</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K57" s="1"/>
       <c r="L57" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D58" s="7">
         <v>433.83</v>
@@ -3398,28 +3392,28 @@
         <v>905.48</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K58" s="1"/>
       <c r="L58" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D59" s="1">
         <v>0</v>
@@ -3430,25 +3424,25 @@
       <c r="F59" s="7"/>
       <c r="G59" s="7"/>
       <c r="H59" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K59" s="1"/>
       <c r="L59" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C60" s="1"/>
       <c r="D60" s="1">
@@ -3462,28 +3456,28 @@
         <v>0.37</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K60" s="1"/>
       <c r="L60" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" ht="58" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D61" s="1">
         <v>70</v>
@@ -3496,25 +3490,25 @@
         <v>100</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K61" s="1"/>
       <c r="L61" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" ht="29" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C62" s="1"/>
       <c r="D62" s="7">
@@ -3528,28 +3522,28 @@
         <v>9</v>
       </c>
       <c r="H62" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K62" s="1"/>
       <c r="L62" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D63" s="8">
         <v>6.7212500000000004</v>
@@ -3560,26 +3554,26 @@
       <c r="F63" s="7"/>
       <c r="G63" s="7"/>
       <c r="H63" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I63" s="1"/>
       <c r="J63" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K63" s="1"/>
       <c r="L63" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D64" s="1">
         <v>0.15</v>
@@ -3594,17 +3588,17 @@
         <v>0.2</v>
       </c>
       <c r="H64" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K64" s="1"/>
       <c r="L64" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -3623,62 +3617,62 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1" t="s">
         <v>76</v>
-      </c>
-      <c r="D1" t="s">
-        <v>77</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2">
         <f xml:space="preserve"> 172*0.3*0.25*0.5</f>
         <v>6.45</v>
       </c>
       <c r="E2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -3688,18 +3682,18 @@
         <v>0.30499999999999999</v>
       </c>
       <c r="E3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -3708,18 +3702,18 @@
         <v>0.1</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -3728,310 +3722,310 @@
         <v>0.1</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>200</v>
       </c>
       <c r="E6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D7">
         <v>200</v>
       </c>
       <c r="E7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" t="s">
         <v>78</v>
-      </c>
-      <c r="B8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" t="s">
-        <v>79</v>
       </c>
       <c r="D8">
         <v>750</v>
       </c>
       <c r="E8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D9">
         <v>6750</v>
       </c>
       <c r="E9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D10">
         <v>2500</v>
       </c>
       <c r="E10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D11">
         <v>200</v>
       </c>
       <c r="E11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D12">
         <v>1000</v>
       </c>
       <c r="E12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D13">
         <v>2000</v>
       </c>
       <c r="E13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D14">
         <v>10</v>
       </c>
       <c r="E14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F14" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D15">
         <v>0.1</v>
       </c>
       <c r="E15" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D16">
         <v>400</v>
       </c>
       <c r="E16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D17">
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F17" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D18">
         <v>1000</v>
       </c>
       <c r="E18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D19">
         <v>3000</v>
       </c>
       <c r="E19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D20">
         <v>40</v>
       </c>
       <c r="E20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -4041,82 +4035,82 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
-  <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
@@ -4125,201 +4119,157 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>139</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>139</v>
       </c>
       <c r="C13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" t="s">
+        <v>139</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>5</v>
       </c>
-      <c r="B14" t="s">
-        <v>140</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B16" t="s">
-        <v>140</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>8</v>
-      </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>48</v>
       </c>
       <c r="C17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>140</v>
+        <v>48</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B19" t="s">
-        <v>140</v>
+        <v>48</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>7</v>
-      </c>
-      <c r="B22" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25">
         <v>0</v>
       </c>
     </row>
@@ -4331,265 +4281,265 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{345A3703-44E3-4DF2-AACF-D4D2788B63CA}">
   <dimension ref="A16:L28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="16" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D16" s="11">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11">
+        <v>0.26</v>
+      </c>
+      <c r="G16" s="11">
+        <v>0.33</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="K16" s="11"/>
+      <c r="L16" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" s="18">
+        <v>0.4</v>
+      </c>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18">
+        <v>0</v>
+      </c>
+      <c r="G17" s="18">
+        <v>1</v>
+      </c>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="J17" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="K17" s="18"/>
+      <c r="L17" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" s="11">
+        <v>0.22</v>
+      </c>
+      <c r="E18" s="11">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="K18" s="11"/>
+      <c r="L18" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="D19" s="18">
+        <v>0.4</v>
+      </c>
+      <c r="E19" s="18">
+        <v>0.8</v>
+      </c>
+      <c r="F19" s="20">
+        <v>0.25</v>
+      </c>
+      <c r="G19" s="20">
+        <v>0.4</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="I19" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="J19" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="K19" s="18"/>
+      <c r="L19" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+      <c r="A25" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B25" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="D25" s="18">
+        <v>0.2</v>
+      </c>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18">
+        <v>0.12</v>
+      </c>
+      <c r="G25" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="I25" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="J25" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="K25" s="18"/>
+      <c r="L25" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D16" s="16">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16">
-        <v>0.26</v>
-      </c>
-      <c r="G16" s="16">
-        <v>0.33</v>
-      </c>
-      <c r="H16" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="17" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="C26" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D26" s="11">
+        <v>0.2</v>
+      </c>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11">
+        <v>0</v>
+      </c>
+      <c r="G26" s="11">
+        <v>1</v>
+      </c>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="J26" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="K26" s="11"/>
+      <c r="L26" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D17" s="19">
-        <v>0.4</v>
-      </c>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19">
-        <v>0</v>
-      </c>
-      <c r="G17" s="19">
-        <v>1</v>
-      </c>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="J17" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="K17" s="19"/>
-      <c r="L17" s="20" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D18" s="16">
-        <v>0.22</v>
-      </c>
-      <c r="E18" s="16">
-        <v>3.5000000000000003E-2</v>
-      </c>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="17" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" ht="105" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D19" s="19">
-        <v>0.4</v>
-      </c>
-      <c r="E19" s="19">
-        <v>0.8</v>
-      </c>
-      <c r="F19" s="21">
-        <v>0.25</v>
-      </c>
-      <c r="G19" s="21">
-        <v>0.4</v>
-      </c>
-      <c r="H19" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="I19" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="J19" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="K19" s="19"/>
-      <c r="L19" s="20" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="60" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D25" s="19">
-        <v>0.2</v>
-      </c>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19">
-        <v>0.12</v>
-      </c>
-      <c r="G25" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="H25" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="I25" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="J25" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="K25" s="19"/>
-      <c r="L25" s="20" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D26" s="16">
-        <v>0.2</v>
-      </c>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16">
-        <v>0</v>
-      </c>
-      <c r="G26" s="16">
-        <v>1</v>
-      </c>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="J26" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="17" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="75" x14ac:dyDescent="0.25">
-      <c r="A27" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D27" s="19">
+      <c r="B27" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C27" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="D27" s="18">
         <v>0.21</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="18">
         <f>0.02</f>
         <v>0.02</v>
       </c>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="K27" s="19"/>
-      <c r="L27" s="20" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="285" x14ac:dyDescent="0.25">
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="K27" s="18"/>
+      <c r="L27" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="261" x14ac:dyDescent="0.35">
       <c r="A28" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D28" s="16">
+        <v>16</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D28" s="11">
         <v>0.2</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28" s="11">
         <v>0.4</v>
       </c>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="I28" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="J28" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="17" t="s">
-        <v>59</v>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="J28" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="K28" s="11"/>
+      <c r="L28" s="16" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed bounds from the scenario spreadsheet. Updated the number of morris trajectories to improve stability.
</commit_message>
<xml_diff>
--- a/Data/scenarios.xlsx
+++ b/Data/scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Documents\GitHub Repos\merging_SFW_decomposition_models\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbuchkow\Documents\GitHubRepos\merging_SFW_decomposition_models\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFA2C65-4279-49A4-B48A-43BF61C2D6F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E142A27D-E6FE-44E6-BE4A-924FBC093872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7C97690C-9E7B-4D0E-86C0-16835BCB4BB0}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -489,7 +489,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1553,20 +1553,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD4418A0-EB93-4361-AE80-4D25DF544368}">
   <dimension ref="A1:L64"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="22.7265625" customWidth="1"/>
-    <col min="4" max="4" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="52.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.75" customWidth="1"/>
+    <col min="4" max="4" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.25" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="13.26953125" customWidth="1"/>
+    <col min="11" max="11" width="13.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="28.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -1620,12 +1620,8 @@
       <c r="E2" s="1">
         <v>0.06</v>
       </c>
-      <c r="F2" s="1">
-        <v>0</v>
-      </c>
-      <c r="G2" s="1">
-        <v>1</v>
-      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
         <v>23</v>
       </c>
@@ -1638,7 +1634,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -1654,12 +1650,8 @@
       <c r="E3" s="1">
         <v>0.06</v>
       </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1</v>
-      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
       <c r="H3" s="1" t="s">
         <v>25</v>
       </c>
@@ -1672,7 +1664,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="28.5">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -1706,7 +1698,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="28.5">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
@@ -1735,7 +1727,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="28.5">
       <c r="A6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1764,7 +1756,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="28.5">
       <c r="A7" s="1" t="s">
         <v>29</v>
       </c>
@@ -1793,7 +1785,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="28.5">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -1828,7 +1820,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" ht="28.5">
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
@@ -1858,7 +1850,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1892,7 +1884,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -1908,12 +1900,8 @@
       <c r="E11" s="1">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-      <c r="G11" s="1">
-        <v>1</v>
-      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
       <c r="H11" s="1" t="s">
         <v>140</v>
       </c>
@@ -1926,7 +1914,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -1964,7 +1952,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12">
       <c r="A13" s="1" t="s">
         <v>18</v>
       </c>
@@ -2002,7 +1990,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -2018,12 +2006,8 @@
       <c r="E14" s="1">
         <v>7.0300000000000001E-2</v>
       </c>
-      <c r="F14" s="1">
-        <v>0</v>
-      </c>
-      <c r="G14" s="1">
-        <v>1</v>
-      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
         <v>27</v>
       </c>
@@ -2036,7 +2020,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -2068,7 +2052,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12">
       <c r="A16" s="1" t="s">
         <v>19</v>
       </c>
@@ -2098,7 +2082,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="28.5">
       <c r="A17" s="1" t="s">
         <v>31</v>
       </c>
@@ -2112,12 +2096,8 @@
         <v>0</v>
       </c>
       <c r="E17" s="1"/>
-      <c r="F17" s="1">
-        <v>0</v>
-      </c>
-      <c r="G17" s="1">
-        <v>1</v>
-      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
         <v>108</v>
@@ -2130,7 +2110,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -2156,7 +2136,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12">
       <c r="A19" s="1" t="s">
         <v>13</v>
       </c>
@@ -2182,7 +2162,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12">
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
@@ -2210,7 +2190,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -2244,7 +2224,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12">
       <c r="A22" s="1" t="s">
         <v>38</v>
       </c>
@@ -2272,7 +2252,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12">
       <c r="A23" s="1" t="s">
         <v>35</v>
       </c>
@@ -2303,7 +2283,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" ht="16.5">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
@@ -2337,7 +2317,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="15.75">
       <c r="A25" s="1" t="s">
         <v>12</v>
       </c>
@@ -2353,12 +2333,8 @@
       <c r="E25" s="1">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F25" s="1">
-        <v>0</v>
-      </c>
-      <c r="G25" s="1">
-        <v>1</v>
-      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
       <c r="H25" s="14" t="s">
         <v>145</v>
       </c>
@@ -2373,7 +2349,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="42.75">
       <c r="A26" s="1" t="s">
         <v>17</v>
       </c>
@@ -2405,7 +2381,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12">
       <c r="A27" s="1" t="s">
         <v>18</v>
       </c>
@@ -2425,7 +2401,7 @@
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12">
       <c r="A28" s="1" t="s">
         <v>37</v>
       </c>
@@ -2453,7 +2429,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12">
       <c r="A29" s="1" t="s">
         <v>14</v>
       </c>
@@ -2487,7 +2463,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12">
       <c r="A30" s="1" t="s">
         <v>19</v>
       </c>
@@ -2519,7 +2495,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" ht="28.5">
       <c r="A31" s="1" t="s">
         <v>40</v>
       </c>
@@ -2549,7 +2525,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" ht="28.5">
       <c r="A32" s="1" t="s">
         <v>41</v>
       </c>
@@ -2579,7 +2555,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" ht="16.5">
       <c r="A33" s="1" t="s">
         <v>11</v>
       </c>
@@ -2609,7 +2585,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" ht="15.75">
       <c r="A34" s="1" t="s">
         <v>13</v>
       </c>
@@ -2637,7 +2613,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" ht="28.5">
       <c r="A35" s="1" t="s">
         <v>36</v>
       </c>
@@ -2667,7 +2643,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12">
       <c r="A36" s="1" t="s">
         <v>20</v>
       </c>
@@ -2701,7 +2677,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" ht="28.5">
       <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
@@ -2729,7 +2705,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" ht="28.5">
       <c r="A38" s="1" t="s">
         <v>35</v>
       </c>
@@ -2760,7 +2736,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
@@ -2790,7 +2766,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" ht="42.75">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
@@ -2806,12 +2782,8 @@
       <c r="E40" s="1">
         <v>0.04</v>
       </c>
-      <c r="F40" s="1">
-        <v>0</v>
-      </c>
-      <c r="G40" s="1">
-        <v>1</v>
-      </c>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
       <c r="H40" s="1" t="s">
         <v>43</v>
       </c>
@@ -2824,7 +2796,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12">
       <c r="A41" s="1" t="s">
         <v>17</v>
       </c>
@@ -2858,7 +2830,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12">
       <c r="A42" s="1" t="s">
         <v>18</v>
       </c>
@@ -2892,7 +2864,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" ht="28.5">
       <c r="A43" s="1" t="s">
         <v>37</v>
       </c>
@@ -2922,7 +2894,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12">
       <c r="A44" s="1" t="s">
         <v>14</v>
       </c>
@@ -2952,7 +2924,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12">
       <c r="A45" s="1" t="s">
         <v>19</v>
       </c>
@@ -2980,7 +2952,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" ht="42.75">
       <c r="A46" s="1" t="s">
         <v>40</v>
       </c>
@@ -3010,7 +2982,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" ht="28.5">
       <c r="A47" s="1" t="s">
         <v>41</v>
       </c>
@@ -3042,7 +3014,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12">
       <c r="A48" s="1" t="s">
         <v>11</v>
       </c>
@@ -3072,7 +3044,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" ht="42.75">
       <c r="A49" s="1" t="s">
         <v>13</v>
       </c>
@@ -3102,7 +3074,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12">
       <c r="A50" s="1" t="s">
         <v>51</v>
       </c>
@@ -3116,12 +3088,8 @@
         <v>0.5</v>
       </c>
       <c r="E50" s="7"/>
-      <c r="F50" s="7">
-        <v>0.5</v>
-      </c>
-      <c r="G50" s="7">
-        <v>0.5</v>
-      </c>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
       <c r="H50" s="1" t="s">
         <v>138</v>
       </c>
@@ -3136,7 +3104,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12">
       <c r="A51" s="1" t="s">
         <v>20</v>
       </c>
@@ -3172,7 +3140,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="52" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" ht="42.75">
       <c r="A52" s="1" t="s">
         <v>49</v>
       </c>
@@ -3208,7 +3176,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="53" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" ht="15.75">
       <c r="A53" s="1" t="s">
         <v>50</v>
       </c>
@@ -3241,7 +3209,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" ht="28.5">
       <c r="A54" s="1" t="s">
         <v>53</v>
       </c>
@@ -3273,7 +3241,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12">
       <c r="A55" s="1" t="s">
         <v>54</v>
       </c>
@@ -3305,7 +3273,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12">
       <c r="A56" s="1" t="s">
         <v>10</v>
       </c>
@@ -3335,7 +3303,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="57" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" ht="42.75">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
@@ -3369,7 +3337,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12">
       <c r="A58" s="1" t="s">
         <v>17</v>
       </c>
@@ -3405,7 +3373,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12">
       <c r="A59" s="1" t="s">
         <v>18</v>
       </c>
@@ -3437,7 +3405,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12">
       <c r="A60" s="1" t="s">
         <v>52</v>
       </c>
@@ -3449,12 +3417,8 @@
         <v>0.37</v>
       </c>
       <c r="E60" s="7"/>
-      <c r="F60" s="7">
-        <v>0.37</v>
-      </c>
-      <c r="G60" s="7">
-        <v>0.37</v>
-      </c>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
       <c r="H60" s="1" t="s">
         <v>138</v>
       </c>
@@ -3469,7 +3433,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" ht="57">
       <c r="A61" s="1" t="s">
         <v>14</v>
       </c>
@@ -3503,7 +3467,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="62" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" ht="42.75">
       <c r="A62" s="1" t="s">
         <v>19</v>
       </c>
@@ -3535,7 +3499,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12">
       <c r="A63" s="1" t="s">
         <v>11</v>
       </c>
@@ -3565,7 +3529,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="64" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" ht="42.75">
       <c r="A64" s="1" t="s">
         <v>13</v>
       </c>
@@ -3617,16 +3581,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA0710C0-AB94-4FBF-AB29-E5085BC4F559}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" customWidth="1"/>
+    <col min="1" max="1" width="11.75" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
+    <col min="3" max="3" width="13.875" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="35.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>74</v>
       </c>
@@ -3646,7 +3610,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -3667,7 +3631,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>77</v>
       </c>
@@ -3688,7 +3652,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>77</v>
       </c>
@@ -3708,7 +3672,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>77</v>
       </c>
@@ -3728,7 +3692,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>77</v>
       </c>
@@ -3748,7 +3712,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>77</v>
       </c>
@@ -3768,7 +3732,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -3788,7 +3752,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -3808,7 +3772,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>77</v>
       </c>
@@ -3828,7 +3792,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>93</v>
       </c>
@@ -3848,7 +3812,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>93</v>
       </c>
@@ -3868,7 +3832,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>93</v>
       </c>
@@ -3888,7 +3852,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>93</v>
       </c>
@@ -3908,7 +3872,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>93</v>
       </c>
@@ -3928,7 +3892,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>93</v>
       </c>
@@ -3948,7 +3912,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>93</v>
       </c>
@@ -3968,7 +3932,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -3988,7 +3952,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>93</v>
       </c>
@@ -4008,7 +3972,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>93</v>
       </c>
@@ -4036,13 +4000,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC182590-26D0-4168-8E7C-B448CD67FE47}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>75</v>
       </c>
@@ -4053,7 +4017,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -4064,7 +4028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -4075,7 +4039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -4086,7 +4050,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4097,7 +4061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -4108,7 +4072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -4119,7 +4083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -4130,7 +4094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -4141,7 +4105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -4152,7 +4116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -4163,7 +4127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -4174,7 +4138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -4185,7 +4149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -4196,7 +4160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -4207,7 +4171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -4218,7 +4182,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -4229,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -4240,7 +4204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -4251,7 +4215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -4262,7 +4226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -4281,9 +4245,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{345A3703-44E3-4DF2-AACF-D4D2788B63CA}">
   <dimension ref="A16:L28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="16" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" ht="71.25">
       <c r="A16" s="15" t="s">
         <v>15</v>
       </c>
@@ -4315,7 +4279,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="28.5">
       <c r="A17" s="17" t="s">
         <v>15</v>
       </c>
@@ -4347,7 +4311,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="57">
       <c r="A18" s="15" t="s">
         <v>15</v>
       </c>
@@ -4377,7 +4341,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="85.5">
       <c r="A19" s="17" t="s">
         <v>15</v>
       </c>
@@ -4413,7 +4377,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="58" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="57">
       <c r="A25" s="17" t="s">
         <v>16</v>
       </c>
@@ -4447,7 +4411,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="28.5">
       <c r="A26" s="15" t="s">
         <v>16</v>
       </c>
@@ -4479,7 +4443,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" ht="71.25">
       <c r="A27" s="17" t="s">
         <v>16</v>
       </c>
@@ -4510,7 +4474,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="261" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" ht="256.5">
       <c r="A28" s="15" t="s">
         <v>16</v>
       </c>

</xml_diff>